<commit_message>
New bee species name.
</commit_message>
<xml_diff>
--- a/Data/Antimicrobial_of_honey.xlsx
+++ b/Data/Antimicrobial_of_honey.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Antimicrobial" sheetId="1" state="visible" r:id="rId2"/>
@@ -98,7 +98,7 @@
     <t xml:space="preserve">M. fuscopilosa FIED001 (7)</t>
   </si>
   <si>
-    <t xml:space="preserve">M. fasciculata RGB004 (6)</t>
+    <t xml:space="preserve">M. grandis RGB004 (6)</t>
   </si>
   <si>
     <t xml:space="preserve">M. fuscopilosa RGY001 (8)</t>
@@ -107,10 +107,10 @@
     <t xml:space="preserve">M. fuscopilosa RIG003 (9)</t>
   </si>
   <si>
-    <t xml:space="preserve">M. fasciculata RIG005 (5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M. fasciculata RYMG001 (4)</t>
+    <t xml:space="preserve">M. grandis RIG005 (5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M. grandis RYMG001 (4)</t>
   </si>
   <si>
     <t xml:space="preserve">T. angustula RYTA006 (1)</t>

</xml_diff>